<commit_message>
Selenium e Playwright com BDD adicionados
</commit_message>
<xml_diff>
--- a/Casos de Teste - BDD.xlsx
+++ b/Casos de Teste - BDD.xlsx
@@ -44,8 +44,10 @@
   </si>
   <si>
     <t xml:space="preserve">Dado que o usuário esteja na tela de login
-Quando o usuário inserir um username não cadastrado
-Então exibir mensagem que username e senha inseridos não combinam com nenhum usuário</t>
+        Quando o usuário inserir um username ainda não cadastrado
+        E o usuário inserir uma senha
+        E apertar em login
+        Então exibir mensagem que username e senha inseridos não combinam com nenhum usuário</t>
   </si>
   <si>
     <t xml:space="preserve">PASSOU</t>
@@ -398,37 +400,37 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="000000"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4285f4"/>
+        <a:srgbClr val="4285F4"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="ea4335"/>
+        <a:srgbClr val="EA4335"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="fbbc04"/>
+        <a:srgbClr val="FBBC04"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="34a853"/>
+        <a:srgbClr val="34A853"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="ff6d01"/>
+        <a:srgbClr val="FF6D01"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="46bdc6"/>
+        <a:srgbClr val="46BDC6"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="1155cc"/>
+        <a:srgbClr val="1155CC"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="1155cc"/>
+        <a:srgbClr val="1155CC"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Sheets">
@@ -595,7 +597,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="77.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
         <v>5</v>
       </c>

</xml_diff>